<commit_message>
modifications in the backend
</commit_message>
<xml_diff>
--- a/final_year.xlsx
+++ b/final_year.xlsx
@@ -827,7 +827,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -844,7 +844,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -861,7 +861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -878,7 +878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>13</v>
       </c>

</xml_diff>